<commit_message>
updating draft MOBEAST figure, includes fDOM prelim analysis
</commit_message>
<xml_diff>
--- a/data/raw_data/DOC/MOBEAST_NPOC_TN_241010.xlsx
+++ b/data/raw_data/DOC/MOBEAST_NPOC_TN_241010.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/keanurochette/Desktop/Git Hub Repository/MOBEAST/data/raw_data/DOC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED480425-A5FD-ED4E-8406-4C02AD87E468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BE2E405-4D84-5943-B50E-EDDEEB75CFDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17300" xr2:uid="{43D7ACD6-8BA2-0A46-89F6-569A470420D9}"/>
+    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="17340" xr2:uid="{43D7ACD6-8BA2-0A46-89F6-569A470420D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>

</xml_diff>